<commit_message>
Project2 자료 status 업데이트
</commit_message>
<xml_diff>
--- a/project_2/project2_project status(C2)xlsx.xlsx
+++ b/project_2/project2_project status(C2)xlsx.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pyostry\workspace\aiffel\ai-data-bootcamp\Project_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06B5C75D-AF26-46AF-BC40-CEF79F2B3CA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42D23758-A6CB-413A-823C-DAB0C3030AE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{5FF54064-7DDC-427B-93D7-EF78D75E5195}"/>
   </bookViews>
@@ -327,9 +327,6 @@
   </si>
   <si>
     <t>H1·H2·H3가 신규·유지·객단가로 매출의 세 축을 빠짐없이 덮는다.</t>
-  </si>
-  <si>
-    <t>가설 트리의 각 가지를 AARRR 어느 단계 지표로 측정할지 매핑한다. HEART, GAME 등 다른 지표 설계 프레임워크를 적용할 수 있다.</t>
   </si>
   <si>
     <r>
@@ -1444,6 +1441,10 @@
     <t>링크</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>가설 트리의 각 가지를 AARRR 어느 단계 지표로 측정할지 매핑한다. HEART, GAME 등 다른 지표 설계 프레임워크를 적용할 수 있다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -1451,7 +1452,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="176" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
-    <numFmt numFmtId="184" formatCode="[$-412]yyyy&quot;년&quot;\ m&quot;월&quot;\ d&quot;일&quot;\ dddd\ h&quot;시&quot;\ mm&quot;분&quot;"/>
+    <numFmt numFmtId="177" formatCode="[$-412]yyyy&quot;년&quot;\ m&quot;월&quot;\ d&quot;일&quot;\ dddd\ h&quot;시&quot;\ mm&quot;분&quot;"/>
   </numFmts>
   <fonts count="23" x14ac:knownFonts="1">
     <font>
@@ -1938,7 +1939,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2053,6 +2054,63 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2060,6 +2118,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2071,65 +2138,41 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2140,35 +2183,8 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2178,27 +2194,6 @@
     </xf>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="184" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -10901,8 +10896,8 @@
   <sheetPr>
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:C136"/>
-  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:C135"/>
+  <sheetFormatPr defaultRowHeight="17" outlineLevelRow="2" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="16.83203125" style="20" customWidth="1"/>
     <col min="2" max="2" width="32.9140625" customWidth="1"/>
@@ -10919,597 +10914,626 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="22" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="A5" s="22" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A6" s="22" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="26" x14ac:dyDescent="0.45">
-      <c r="A8" s="21" t="s">
+    <row r="6" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="7" spans="1:1" ht="26" collapsed="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="21" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A8" s="20" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A9" s="20" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A10" s="20" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="12" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A12" s="22" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="14" spans="1:1" ht="21" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A14" s="23" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="24" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="17" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="25" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A18" s="25" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A19" s="25" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A20" s="25" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A21" s="25" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A22" s="25" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A23" s="25" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A24" s="25" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A25" s="25" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A26" s="25" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A27" s="25" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="29" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A29" s="22" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A30" s="20" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A31" s="20" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A32" s="20" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="34" spans="1:1" ht="26" collapsed="1" x14ac:dyDescent="0.45">
+      <c r="A34" s="21" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A9" s="20" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A10" s="20" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A11" s="20" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A13" s="22" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" ht="21" x14ac:dyDescent="0.45">
-      <c r="A15" s="23" t="s">
+    <row r="35" spans="1:1" hidden="1" outlineLevel="2" x14ac:dyDescent="0.45">
+      <c r="A35" s="20" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" hidden="1" outlineLevel="2" x14ac:dyDescent="0.45">
+      <c r="A36" s="22" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" hidden="1" outlineLevel="2" x14ac:dyDescent="0.45">
+      <c r="A37" s="20" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" hidden="1" outlineLevel="2" x14ac:dyDescent="0.45"/>
+    <row r="39" spans="1:1" hidden="1" outlineLevel="2" x14ac:dyDescent="0.45">
+      <c r="A39" s="22" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" hidden="1" outlineLevel="2" x14ac:dyDescent="0.45"/>
+    <row r="41" spans="1:1" ht="26" collapsed="1" x14ac:dyDescent="0.45">
+      <c r="A41" s="21" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A42" s="20" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A43" s="20" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A44" s="20" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="46" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A46" s="22" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="48" spans="1:1" ht="21" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A48" s="23" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A16" s="24" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A18" s="25" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A19" s="25" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A20" s="25" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A21" s="25" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A22" s="25" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A23" s="25" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A24" s="25" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A25" s="25" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A26" s="25" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A27" s="25" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A28" s="25" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A30" s="22" t="s">
+    <row r="49" spans="1:3" ht="21" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A49" s="23" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A50" s="26"/>
+      <c r="B50" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="C50" s="17" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A51" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="B51" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="C51" s="18" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A52" s="27" t="s">
+        <v>82</v>
+      </c>
+      <c r="B52" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="C52" s="18" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A53" s="27" t="s">
+        <v>85</v>
+      </c>
+      <c r="B53" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="C53" s="18" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A54" s="27" t="s">
+        <v>88</v>
+      </c>
+      <c r="B54" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="C54" s="18" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A55" s="27" t="s">
+        <v>91</v>
+      </c>
+      <c r="B55" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="C55" s="18" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="57" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A57" s="22" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A58" s="24" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="60" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A60" s="25" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A61" s="25" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A62" s="25" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A63" s="25" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A64" s="25" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A65" s="25" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A66" s="25" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A67" s="25" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A68" s="25" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A69" s="25" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A70" s="25" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A71" s="25" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A72" s="25" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A73" s="25" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="75" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A75" s="22" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A31" s="20" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A32" s="20" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A33" s="20" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" ht="26" x14ac:dyDescent="0.45">
-      <c r="A36" s="21" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A37" s="20" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A38" s="22" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A39" s="20" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A41" s="22" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" ht="26" x14ac:dyDescent="0.45">
-      <c r="A43" s="21" t="s">
+    <row r="76" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A76" s="20" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A77" s="20" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A78" s="20" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="80" spans="1:1" ht="21" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A80" s="23" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A81" s="22" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A82" s="22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A83" s="22" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A84" s="20" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="86" spans="1:1" ht="26" collapsed="1" x14ac:dyDescent="0.45">
+      <c r="A86" s="21" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A44" s="20" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A45" s="20" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A46" s="20" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A48" s="22" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" ht="21" x14ac:dyDescent="0.45">
-      <c r="A50" s="23" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" ht="21" x14ac:dyDescent="0.45">
-      <c r="A51" s="23" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A52" s="26"/>
-      <c r="B52" s="17" t="s">
-        <v>78</v>
-      </c>
-      <c r="C52" s="17" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A53" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="B53" s="18" t="s">
-        <v>81</v>
-      </c>
-      <c r="C53" s="18" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A54" s="27" t="s">
-        <v>83</v>
-      </c>
-      <c r="B54" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="C54" s="18" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A55" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="B55" s="18" t="s">
-        <v>87</v>
-      </c>
-      <c r="C55" s="18" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A56" s="27" t="s">
-        <v>89</v>
-      </c>
-      <c r="B56" s="18" t="s">
-        <v>90</v>
-      </c>
-      <c r="C56" s="18" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A57" s="27" t="s">
-        <v>92</v>
-      </c>
-      <c r="B57" s="18" t="s">
-        <v>93</v>
-      </c>
-      <c r="C57" s="18" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A59" s="22" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A60" s="24" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A62" s="25" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A63" s="25" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A64" s="25" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A65" s="25" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A66" s="25" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A67" s="25" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A68" s="25" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A69" s="25" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A70" s="25" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A71" s="25" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A72" s="25" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A73" s="25" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A74" s="25" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A75" s="25" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A77" s="22" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A78" s="20" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A79" s="20" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A80" s="20" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="82" spans="1:1" ht="21" x14ac:dyDescent="0.45">
-      <c r="A82" s="23" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A83" s="22" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A84" s="22" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A85" s="22" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A86" s="20" t="s">
+    <row r="87" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A87" s="20" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="88" spans="1:1" ht="26" x14ac:dyDescent="0.45">
-      <c r="A88" s="21" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A88" s="20" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="A89" s="20" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A90" s="20" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A91" s="20" t="s">
+    <row r="90" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="91" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A91" s="22" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A93" s="22" t="s">
+    <row r="92" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="93" spans="1:1" ht="26" collapsed="1" x14ac:dyDescent="0.45">
+      <c r="A93" s="21" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="95" spans="1:1" ht="26" x14ac:dyDescent="0.45">
-      <c r="A95" s="21" t="s">
+    <row r="94" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A94" s="20" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A95" s="20" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="A96" s="20" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A97" s="20" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A98" s="20" t="s">
+    <row r="97" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="98" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A98" s="22" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A100" s="22" t="s">
+    <row r="99" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="100" spans="1:3" ht="26" collapsed="1" x14ac:dyDescent="0.45">
+      <c r="A100" s="21" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="102" spans="1:1" ht="26" x14ac:dyDescent="0.45">
-      <c r="A102" s="21" t="s">
+    <row r="101" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A101" s="20" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A103" s="20" t="s">
+    <row r="102" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A102" s="20" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A104" s="20" t="s">
+    <row r="103" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="104" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A104" s="22" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A106" s="22" t="s">
+    <row r="105" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="106" spans="1:3" ht="26" collapsed="1" x14ac:dyDescent="0.45">
+      <c r="A106" s="21" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="108" spans="1:1" ht="26" x14ac:dyDescent="0.45">
-      <c r="A108" s="21" t="s">
+    <row r="107" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="108" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A108" s="20" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A110" s="20" t="s">
+    <row r="109" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="110" spans="1:3" ht="21" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A110" s="23" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="112" spans="1:1" ht="21" x14ac:dyDescent="0.45">
-      <c r="A112" s="23" t="s">
+    <row r="111" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="112" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A112" s="26" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A114" s="26" t="s">
+      <c r="B112" s="17" t="s">
         <v>134</v>
       </c>
-      <c r="B114" s="17" t="s">
+      <c r="C112" s="17" t="s">
         <v>135</v>
       </c>
-      <c r="C114" s="17" t="s">
+    </row>
+    <row r="113" spans="1:3" ht="34" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A113" s="27" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="115" spans="1:3" ht="34" x14ac:dyDescent="0.45">
-      <c r="A115" s="27" t="s">
+      <c r="B113" s="18" t="s">
         <v>137</v>
       </c>
-      <c r="B115" s="18" t="s">
+      <c r="C113" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="C115" s="18" t="s">
+    </row>
+    <row r="114" spans="1:3" ht="51" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A114" s="27" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="116" spans="1:3" ht="51" x14ac:dyDescent="0.45">
-      <c r="A116" s="27" t="s">
+      <c r="B114" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="B116" s="18" t="s">
+      <c r="C114" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="C116" s="18" t="s">
+    </row>
+    <row r="115" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="116" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A116" s="20" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="118" spans="1:3" ht="21" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A118" s="23" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A118" s="20" t="s">
+    <row r="119" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A119" s="20" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A120" s="20" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A121" s="20" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A122" s="20" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="124" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A124" s="22" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45"/>
+    <row r="126" spans="1:3" ht="21" collapsed="1" x14ac:dyDescent="0.45">
+      <c r="A126" s="23" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A127" s="30" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="120" spans="1:3" ht="21" x14ac:dyDescent="0.45">
-      <c r="A120" s="23" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A121" s="20" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A122" s="20" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A123" s="20" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A124" s="20" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A126" s="22" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="128" spans="1:3" ht="21" x14ac:dyDescent="0.45">
-      <c r="A128" s="23" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A129" s="30" t="s">
+      <c r="B127" s="28" t="s">
         <v>150</v>
       </c>
-      <c r="B129" s="28" t="s">
+    </row>
+    <row r="128" spans="1:3" ht="34" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A128" s="31" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="130" spans="1:2" ht="34" x14ac:dyDescent="0.45">
+      <c r="B128" s="29" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" ht="51" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
+      <c r="A129" s="31" t="s">
+        <v>153</v>
+      </c>
+      <c r="B129" s="29" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" ht="34" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="A130" s="31" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B130" s="29" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="131" spans="1:2" ht="51" x14ac:dyDescent="0.45">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" ht="51" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="A131" s="31" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B131" s="29" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="132" spans="1:2" ht="34" x14ac:dyDescent="0.45">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" ht="34" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="A132" s="31" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B132" s="29" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="133" spans="1:2" ht="51" x14ac:dyDescent="0.45">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" ht="34" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="A133" s="31" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B133" s="29" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="134" spans="1:2" ht="34" x14ac:dyDescent="0.45">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" ht="34" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="A134" s="31" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B134" s="29" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="135" spans="1:2" ht="34" x14ac:dyDescent="0.45">
-      <c r="A135" s="31" t="s">
-        <v>162</v>
-      </c>
-      <c r="B135" s="29" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="136" spans="1:2" ht="34" x14ac:dyDescent="0.45">
-      <c r="A136" s="31" t="s">
         <v>164</v>
       </c>
-      <c r="B136" s="29" t="s">
-        <v>165</v>
-      </c>
-    </row>
+    </row>
+    <row r="135" spans="1:2" collapsed="1" x14ac:dyDescent="0.45"/>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11541,39 +11565,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="38" t="s">
+        <v>167</v>
+      </c>
+      <c r="B1" s="38" t="s">
         <v>168</v>
       </c>
-      <c r="B1" s="44" t="s">
+      <c r="C1" s="38" t="s">
         <v>169</v>
       </c>
-      <c r="C1" s="44" t="s">
+      <c r="D1" s="38" t="s">
         <v>170</v>
-      </c>
-      <c r="D1" s="44" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="85" x14ac:dyDescent="0.45">
       <c r="A2" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="86" t="s">
-        <v>172</v>
+      <c r="B2" s="56" t="s">
+        <v>171</v>
       </c>
       <c r="C2" s="35">
         <v>46274</v>
       </c>
       <c r="D2" s="27" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="34" x14ac:dyDescent="0.45">
       <c r="A3" s="34" t="s">
-        <v>175</v>
-      </c>
-      <c r="B3" s="86" t="s">
-        <v>318</v>
+        <v>174</v>
+      </c>
+      <c r="B3" s="56" t="s">
+        <v>317</v>
       </c>
       <c r="C3" s="35">
         <v>46274</v>
@@ -11582,10 +11606,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" s="33" t="s">
-        <v>173</v>
-      </c>
-      <c r="B4" s="86" t="s">
-        <v>318</v>
+        <v>172</v>
+      </c>
+      <c r="B4" s="56" t="s">
+        <v>317</v>
       </c>
       <c r="C4" s="35">
         <v>46274</v>
@@ -11594,7 +11618,7 @@
     </row>
     <row r="5" spans="1:4" ht="34" x14ac:dyDescent="0.45">
       <c r="A5" s="34" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B5" s="33"/>
       <c r="C5" s="35">
@@ -11604,7 +11628,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" s="33" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B6" s="33"/>
       <c r="C6" s="35">
@@ -11614,7 +11638,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" s="33" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B7" s="33"/>
       <c r="C7" s="35">
@@ -11624,7 +11648,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" s="33" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B8" s="33"/>
       <c r="C8" s="35">
@@ -11634,7 +11658,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A9" s="33" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B9" s="33"/>
       <c r="C9" s="35">
@@ -11644,10 +11668,10 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A10" s="33" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B10" s="33"/>
-      <c r="C10" s="85">
+      <c r="C10" s="55">
         <v>46279.645833333336</v>
       </c>
       <c r="D10" s="33"/>
@@ -11683,30 +11707,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="45" t="s">
+      <c r="B1" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="45" t="s">
+      <c r="C1" s="39" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="45" t="s">
+      <c r="D1" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="E1" s="45" t="s">
+      <c r="E1" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="F1" s="45" t="s">
+      <c r="F1" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="45" t="s">
+      <c r="G1" s="39" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="57" t="s">
         <v>18</v>
       </c>
       <c r="B2" s="7" t="s">
@@ -11723,7 +11747,7 @@
       <c r="G2" s="10"/>
     </row>
     <row r="3" spans="1:7" ht="64" x14ac:dyDescent="0.45">
-      <c r="A3" s="39"/>
+      <c r="A3" s="58"/>
       <c r="B3" s="4" t="s">
         <v>1</v>
       </c>
@@ -11740,9 +11764,9 @@
       <c r="G3" s="11"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A4" s="39"/>
+      <c r="A4" s="58"/>
       <c r="B4" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>29</v>
@@ -11755,7 +11779,7 @@
       <c r="G4" s="11"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A5" s="39"/>
+      <c r="A5" s="58"/>
       <c r="B5" s="4" t="s">
         <v>2</v>
       </c>
@@ -11770,7 +11794,7 @@
       <c r="G5" s="11"/>
     </row>
     <row r="6" spans="1:7" ht="48" x14ac:dyDescent="0.45">
-      <c r="A6" s="39"/>
+      <c r="A6" s="58"/>
       <c r="B6" s="4" t="s">
         <v>3</v>
       </c>
@@ -11789,7 +11813,7 @@
       </c>
     </row>
     <row r="7" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A7" s="40"/>
+      <c r="A7" s="59"/>
       <c r="B7" s="13" t="s">
         <v>15</v>
       </c>
@@ -11800,13 +11824,13 @@
         <v>14</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F7" s="14"/>
       <c r="G7" s="15"/>
     </row>
     <row r="8" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A8" s="46" t="s">
+      <c r="A8" s="60" t="s">
         <v>19</v>
       </c>
       <c r="B8" s="7" t="s">
@@ -11823,11 +11847,11 @@
         <v>36</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A9" s="47"/>
+      <c r="A9" s="61"/>
       <c r="B9" s="4" t="s">
         <v>6</v>
       </c>
@@ -11840,11 +11864,11 @@
       <c r="E9" s="5"/>
       <c r="F9" s="3"/>
       <c r="G9" s="10" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A10" s="47"/>
+      <c r="A10" s="61"/>
       <c r="B10" s="4" t="s">
         <v>4</v>
       </c>
@@ -11855,13 +11879,13 @@
         <v>14</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="11"/>
     </row>
     <row r="11" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A11" s="47"/>
+      <c r="A11" s="61"/>
       <c r="B11" s="4" t="s">
         <v>7</v>
       </c>
@@ -11876,7 +11900,7 @@
       <c r="G11" s="11"/>
     </row>
     <row r="12" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A12" s="48"/>
+      <c r="A12" s="62"/>
       <c r="B12" s="16" t="s">
         <v>8</v>
       </c>
@@ -11889,11 +11913,11 @@
       <c r="E12" s="13"/>
       <c r="F12" s="14"/>
       <c r="G12" s="10" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A13" s="41" t="s">
+      <c r="A13" s="63" t="s">
         <v>20</v>
       </c>
       <c r="B13" s="7" t="s">
@@ -11906,15 +11930,15 @@
         <v>14</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F13" s="9"/>
       <c r="G13" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="64.5" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A14" s="42"/>
+      <c r="A14" s="64"/>
       <c r="B14" s="4" t="s">
         <v>10</v>
       </c>
@@ -11931,9 +11955,9 @@
       <c r="G14" s="11"/>
     </row>
     <row r="15" spans="1:7" ht="64" x14ac:dyDescent="0.45">
-      <c r="A15" s="42"/>
+      <c r="A15" s="64"/>
       <c r="B15" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>45</v>
@@ -11942,17 +11966,17 @@
         <v>13</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>41</v>
       </c>
       <c r="G15" s="12" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="32.5" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A16" s="43"/>
+      <c r="A16" s="65"/>
       <c r="B16" s="16" t="s">
         <v>11</v>
       </c>
@@ -11964,8 +11988,8 @@
       </c>
       <c r="E16" s="13"/>
       <c r="F16" s="14"/>
-      <c r="G16" s="52" t="s">
-        <v>225</v>
+      <c r="G16" s="42" t="s">
+        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -11984,7 +12008,7 @@
   <sheetPr>
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
@@ -11994,194 +12018,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A1" s="50"/>
-      <c r="B1" s="49" t="s">
+      <c r="A1" s="41"/>
+      <c r="B1" s="40" t="s">
+        <v>200</v>
+      </c>
+      <c r="C1" s="40" t="s">
         <v>201</v>
       </c>
-      <c r="C1" s="49" t="s">
+      <c r="D1" s="40" t="s">
         <v>202</v>
       </c>
-      <c r="D1" s="49" t="s">
+    </row>
+    <row r="2" spans="1:4" ht="32" x14ac:dyDescent="0.45">
+      <c r="A2" s="40" t="s">
+        <v>180</v>
+      </c>
+      <c r="B2" s="36" t="s">
+        <v>182</v>
+      </c>
+      <c r="C2" s="37" t="s">
+        <v>188</v>
+      </c>
+      <c r="D2" s="37" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="64" x14ac:dyDescent="0.45">
+      <c r="A3" s="40" t="s">
+        <v>181</v>
+      </c>
+      <c r="B3" s="37" t="s">
+        <v>183</v>
+      </c>
+      <c r="C3" s="37" t="s">
+        <v>189</v>
+      </c>
+      <c r="D3" s="37" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="32" x14ac:dyDescent="0.45">
-      <c r="A2" s="49" t="s">
-        <v>181</v>
-      </c>
-      <c r="B2" s="36" t="s">
-        <v>183</v>
-      </c>
-      <c r="C2" s="37" t="s">
-        <v>189</v>
-      </c>
-      <c r="D2" s="37" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="64" x14ac:dyDescent="0.45">
-      <c r="A3" s="49" t="s">
-        <v>182</v>
-      </c>
-      <c r="B3" s="37" t="s">
-        <v>184</v>
-      </c>
-      <c r="C3" s="37" t="s">
-        <v>190</v>
-      </c>
-      <c r="D3" s="37" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A4" s="51"/>
-      <c r="B4" s="51"/>
-      <c r="C4" s="51"/>
-      <c r="D4" s="51"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A5" s="51"/>
-      <c r="B5" s="51"/>
-      <c r="C5" s="51"/>
-      <c r="D5" s="51"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A6" s="51"/>
-      <c r="B6" s="51"/>
-      <c r="C6" s="51"/>
-      <c r="D6" s="51"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A7" s="51"/>
-      <c r="B7" s="51"/>
-      <c r="C7" s="51"/>
-      <c r="D7" s="51"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A8" s="51"/>
-      <c r="B8" s="51"/>
-      <c r="C8" s="51"/>
-      <c r="D8" s="51"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A9" s="51"/>
-      <c r="B9" s="51"/>
-      <c r="C9" s="51"/>
-      <c r="D9" s="51"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A10" s="51"/>
-      <c r="B10" s="51"/>
-      <c r="C10" s="51"/>
-      <c r="D10" s="51"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A11" s="51"/>
-      <c r="B11" s="51"/>
-      <c r="C11" s="51"/>
-      <c r="D11" s="51"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A12" s="51"/>
-      <c r="B12" s="51"/>
-      <c r="C12" s="51"/>
-      <c r="D12" s="51"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A13" s="51"/>
-      <c r="B13" s="51"/>
-      <c r="C13" s="51"/>
-      <c r="D13" s="51"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A14" s="51"/>
-      <c r="B14" s="51"/>
-      <c r="C14" s="51"/>
-      <c r="D14" s="51"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A15" s="51"/>
-      <c r="B15" s="51"/>
-      <c r="C15" s="51"/>
-      <c r="D15" s="51"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A16" s="51"/>
-      <c r="B16" s="51"/>
-      <c r="C16" s="51"/>
-      <c r="D16" s="51"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A17" s="51"/>
-      <c r="B17" s="51"/>
-      <c r="C17" s="51"/>
-      <c r="D17" s="51"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A18" s="51"/>
-      <c r="B18" s="51"/>
-      <c r="C18" s="51"/>
-      <c r="D18" s="51"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A19" s="51"/>
-      <c r="B19" s="51"/>
-      <c r="C19" s="51"/>
-      <c r="D19" s="51"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A20" s="51"/>
-      <c r="B20" s="51"/>
-      <c r="C20" s="51"/>
-      <c r="D20" s="51"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A21" s="51"/>
-      <c r="B21" s="51"/>
-      <c r="C21" s="51"/>
-      <c r="D21" s="51"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A22" s="51"/>
-      <c r="B22" s="51"/>
-      <c r="C22" s="51"/>
-      <c r="D22" s="51"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A23" s="51"/>
-      <c r="B23" s="51"/>
-      <c r="C23" s="51"/>
-      <c r="D23" s="51"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A24" s="51"/>
-      <c r="B24" s="51"/>
-      <c r="C24" s="51"/>
-      <c r="D24" s="51"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A25" s="51"/>
-      <c r="B25" s="51"/>
-      <c r="C25" s="51"/>
-      <c r="D25" s="51"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A26" s="51"/>
-      <c r="B26" s="51"/>
-      <c r="C26" s="51"/>
-      <c r="D26" s="51"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A27" s="51"/>
-      <c r="B27" s="51"/>
-      <c r="C27" s="51"/>
-      <c r="D27" s="51"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A28" s="51"/>
-      <c r="B28" s="51"/>
-      <c r="C28" s="51"/>
-      <c r="D28" s="51"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -12198,575 +12072,575 @@
   <dimension ref="A1:E75"/>
   <sheetFormatPr defaultRowHeight="16" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="32.58203125" style="57" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.1640625" style="57" customWidth="1"/>
-    <col min="3" max="3" width="57.9140625" style="57" customWidth="1"/>
-    <col min="4" max="4" width="16.08203125" style="57" customWidth="1"/>
-    <col min="5" max="5" width="17.08203125" style="57" customWidth="1"/>
-    <col min="6" max="16384" width="8.6640625" style="57"/>
+    <col min="1" max="1" width="32.58203125" style="45" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.1640625" style="45" customWidth="1"/>
+    <col min="3" max="3" width="57.9140625" style="45" customWidth="1"/>
+    <col min="4" max="4" width="16.08203125" style="45" customWidth="1"/>
+    <col min="5" max="5" width="17.08203125" style="45" customWidth="1"/>
+    <col min="6" max="16384" width="8.6640625" style="45"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="40" t="s">
+        <v>195</v>
+      </c>
+      <c r="B1" s="40" t="s">
         <v>196</v>
       </c>
-      <c r="B1" s="49" t="s">
+      <c r="C1" s="40" t="s">
         <v>197</v>
       </c>
-      <c r="C1" s="49" t="s">
-        <v>198</v>
-      </c>
-      <c r="D1" s="49" t="s">
-        <v>316</v>
+      <c r="D1" s="40" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" s="36" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B2" s="36" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C2" s="36" t="s">
-        <v>235</v>
-      </c>
-      <c r="D2" s="70" t="s">
-        <v>317</v>
+        <v>234</v>
+      </c>
+      <c r="D2" s="50" t="s">
+        <v>316</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="64" x14ac:dyDescent="0.45">
       <c r="A3" s="36" t="s">
-        <v>191</v>
-      </c>
-      <c r="B3" s="58" t="s">
+        <v>190</v>
+      </c>
+      <c r="B3" s="46" t="s">
+        <v>232</v>
+      </c>
+      <c r="C3" s="37" t="s">
+        <v>199</v>
+      </c>
+      <c r="D3" s="50" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A5" s="73" t="s">
+        <v>288</v>
+      </c>
+      <c r="B5" s="73"/>
+      <c r="C5" s="73"/>
+    </row>
+    <row r="6" spans="1:4" ht="32" x14ac:dyDescent="0.45">
+      <c r="A6" s="75" t="s">
+        <v>205</v>
+      </c>
+      <c r="B6" s="47" t="s">
+        <v>206</v>
+      </c>
+      <c r="C6" s="48" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="32" x14ac:dyDescent="0.45">
+      <c r="A7" s="76"/>
+      <c r="B7" s="47" t="s">
+        <v>308</v>
+      </c>
+      <c r="C7" s="48" t="s">
         <v>233</v>
       </c>
-      <c r="C3" s="37" t="s">
-        <v>200</v>
-      </c>
-      <c r="D3" s="70" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A5" s="59" t="s">
+    </row>
+    <row r="8" spans="1:4" ht="32" x14ac:dyDescent="0.45">
+      <c r="A8" s="76"/>
+      <c r="B8" s="47" t="s">
+        <v>311</v>
+      </c>
+      <c r="C8" s="48" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A9" s="76"/>
+      <c r="B9" s="47" t="s">
+        <v>207</v>
+      </c>
+      <c r="C9" s="48" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A10" s="77"/>
+      <c r="B10" s="47" t="s">
+        <v>313</v>
+      </c>
+      <c r="C10" s="48" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A11" s="54" t="s">
+        <v>309</v>
+      </c>
+      <c r="B11" s="47" t="s">
+        <v>208</v>
+      </c>
+      <c r="C11" s="48" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="C12" s="49"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A13" s="67" t="s">
         <v>289</v>
       </c>
-      <c r="B5" s="59"/>
-      <c r="C5" s="59"/>
-    </row>
-    <row r="6" spans="1:4" ht="32" x14ac:dyDescent="0.45">
-      <c r="A6" s="82" t="s">
-        <v>206</v>
-      </c>
-      <c r="B6" s="61" t="s">
-        <v>207</v>
-      </c>
-      <c r="C6" s="62" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="32" x14ac:dyDescent="0.45">
-      <c r="A7" s="83"/>
-      <c r="B7" s="61" t="s">
-        <v>309</v>
-      </c>
-      <c r="C7" s="62" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="32" x14ac:dyDescent="0.45">
-      <c r="A8" s="83"/>
-      <c r="B8" s="61" t="s">
-        <v>312</v>
-      </c>
-      <c r="C8" s="62" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A9" s="83"/>
-      <c r="B9" s="61" t="s">
-        <v>208</v>
-      </c>
-      <c r="C9" s="62" t="s">
+      <c r="B13" s="68"/>
+      <c r="C13" s="69"/>
+    </row>
+    <row r="14" spans="1:4" ht="52" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A14" s="78" t="s">
+        <v>235</v>
+      </c>
+      <c r="B14" s="79"/>
+      <c r="C14" s="80"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A19" s="49"/>
+      <c r="C19" s="49"/>
+      <c r="D19" s="49"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A31" s="73" t="s">
+        <v>290</v>
+      </c>
+      <c r="B31" s="73"/>
+      <c r="C31" s="73"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A32" s="70" t="s">
+        <v>210</v>
+      </c>
+      <c r="B32" s="71"/>
+      <c r="C32" s="72"/>
+    </row>
+    <row r="33" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A33" s="66" t="s">
+        <v>236</v>
+      </c>
+      <c r="B33" s="50" t="s">
+        <v>211</v>
+      </c>
+      <c r="C33" s="74" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A34" s="66"/>
+      <c r="B34" s="50" t="s">
+        <v>212</v>
+      </c>
+      <c r="C34" s="74"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A35" s="66"/>
+      <c r="B35" s="50" t="s">
+        <v>213</v>
+      </c>
+      <c r="C35" s="74"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A36" s="66"/>
+      <c r="B36" s="50" t="s">
+        <v>214</v>
+      </c>
+      <c r="C36" s="74"/>
+    </row>
+    <row r="37" spans="1:5" ht="32" x14ac:dyDescent="0.45">
+      <c r="A37" s="66"/>
+      <c r="B37" s="48" t="s">
+        <v>216</v>
+      </c>
+      <c r="C37" s="74"/>
+    </row>
+    <row r="38" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A38" s="66" t="s">
+        <v>237</v>
+      </c>
+      <c r="B38" s="50" t="s">
+        <v>217</v>
+      </c>
+      <c r="C38" s="74" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A39" s="66"/>
+      <c r="B39" s="50" t="s">
+        <v>218</v>
+      </c>
+      <c r="C39" s="74"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A40" s="66"/>
+      <c r="B40" s="50" t="s">
+        <v>219</v>
+      </c>
+      <c r="C40" s="74"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A42" s="67" t="s">
+        <v>287</v>
+      </c>
+      <c r="B42" s="68"/>
+      <c r="C42" s="69"/>
+    </row>
+    <row r="43" spans="1:5" ht="53" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A43" s="66" t="s">
+        <v>221</v>
+      </c>
+      <c r="B43" s="66"/>
+      <c r="C43" s="66"/>
+    </row>
+    <row r="44" spans="1:5" ht="50.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A44" s="66" t="s">
+        <v>222</v>
+      </c>
+      <c r="B44" s="66"/>
+      <c r="C44" s="66"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A46" s="73" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A10" s="84"/>
-      <c r="B10" s="61" t="s">
-        <v>314</v>
-      </c>
-      <c r="C10" s="62" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A11" s="81" t="s">
-        <v>310</v>
-      </c>
-      <c r="B11" s="61" t="s">
-        <v>209</v>
-      </c>
-      <c r="C11" s="62" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="C12" s="63"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A13" s="72" t="s">
-        <v>290</v>
-      </c>
-      <c r="B13" s="73"/>
-      <c r="C13" s="74"/>
-    </row>
-    <row r="14" spans="1:4" ht="52" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="64" t="s">
-        <v>236</v>
-      </c>
-      <c r="B14" s="65"/>
-      <c r="C14" s="66"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A19" s="63"/>
-      <c r="C19" s="63"/>
-      <c r="D19" s="63"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A31" s="59" t="s">
+      <c r="B46" s="73"/>
+      <c r="C46" s="73"/>
+      <c r="D46" s="73"/>
+      <c r="E46" s="73"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A47" s="44" t="s">
+        <v>238</v>
+      </c>
+      <c r="B47" s="44" t="s">
+        <v>247</v>
+      </c>
+      <c r="C47" s="44" t="s">
+        <v>248</v>
+      </c>
+      <c r="D47" s="44" t="s">
+        <v>249</v>
+      </c>
+      <c r="E47" s="44" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="32" x14ac:dyDescent="0.45">
+      <c r="A48" s="43" t="s">
+        <v>251</v>
+      </c>
+      <c r="B48" s="43" t="s">
+        <v>239</v>
+      </c>
+      <c r="C48" s="43" t="s">
+        <v>252</v>
+      </c>
+      <c r="D48" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="E48" s="43" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="32" x14ac:dyDescent="0.45">
+      <c r="A49" s="43" t="s">
+        <v>253</v>
+      </c>
+      <c r="B49" s="43" t="s">
+        <v>242</v>
+      </c>
+      <c r="C49" s="43" t="s">
+        <v>254</v>
+      </c>
+      <c r="D49" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="E49" s="43" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="48" x14ac:dyDescent="0.45">
+      <c r="A50" s="43" t="s">
+        <v>255</v>
+      </c>
+      <c r="B50" s="43" t="s">
+        <v>242</v>
+      </c>
+      <c r="C50" s="43" t="s">
+        <v>256</v>
+      </c>
+      <c r="D50" s="43" t="s">
+        <v>243</v>
+      </c>
+      <c r="E50" s="43" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="32" x14ac:dyDescent="0.45">
+      <c r="A51" s="43" t="s">
+        <v>258</v>
+      </c>
+      <c r="B51" s="43" t="s">
+        <v>244</v>
+      </c>
+      <c r="C51" s="43" t="s">
+        <v>259</v>
+      </c>
+      <c r="D51" s="43" t="s">
+        <v>245</v>
+      </c>
+      <c r="E51" s="43" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="32" x14ac:dyDescent="0.45">
+      <c r="A52" s="43" t="s">
+        <v>260</v>
+      </c>
+      <c r="B52" s="43" t="s">
+        <v>244</v>
+      </c>
+      <c r="C52" s="43" t="s">
+        <v>261</v>
+      </c>
+      <c r="D52" s="43" t="s">
+        <v>245</v>
+      </c>
+      <c r="E52" s="43" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="32" x14ac:dyDescent="0.45">
+      <c r="A53" s="43" t="s">
+        <v>262</v>
+      </c>
+      <c r="B53" s="43" t="s">
+        <v>244</v>
+      </c>
+      <c r="C53" s="43" t="s">
+        <v>263</v>
+      </c>
+      <c r="D53" s="43" t="s">
+        <v>246</v>
+      </c>
+      <c r="E53" s="43" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A54" s="43" t="s">
+        <v>264</v>
+      </c>
+      <c r="B54" s="43" t="s">
+        <v>244</v>
+      </c>
+      <c r="C54" s="43" t="s">
+        <v>265</v>
+      </c>
+      <c r="D54" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="E54" s="43" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="32" x14ac:dyDescent="0.45">
+      <c r="A55" s="43" t="s">
+        <v>266</v>
+      </c>
+      <c r="B55" s="43" t="s">
+        <v>244</v>
+      </c>
+      <c r="C55" s="43" t="s">
+        <v>267</v>
+      </c>
+      <c r="D55" s="43" t="s">
+        <v>246</v>
+      </c>
+      <c r="E55" s="43" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="48" x14ac:dyDescent="0.45">
+      <c r="A56" s="43"/>
+      <c r="B56" s="43" t="s">
+        <v>269</v>
+      </c>
+      <c r="C56" s="43" t="s">
+        <v>271</v>
+      </c>
+      <c r="D56" s="43" t="s">
+        <v>272</v>
+      </c>
+      <c r="E56" s="51" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="48" x14ac:dyDescent="0.45">
+      <c r="A57" s="43"/>
+      <c r="B57" s="43" t="s">
+        <v>270</v>
+      </c>
+      <c r="C57" s="43" t="s">
+        <v>273</v>
+      </c>
+      <c r="D57" s="43" t="s">
+        <v>274</v>
+      </c>
+      <c r="E57" s="51" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A59" s="82" t="s">
         <v>291</v>
       </c>
-      <c r="B31" s="59"/>
-      <c r="C31" s="59"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A32" s="67" t="s">
-        <v>211</v>
-      </c>
-      <c r="B32" s="68"/>
-      <c r="C32" s="69"/>
-    </row>
-    <row r="33" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="60" t="s">
-        <v>237</v>
-      </c>
-      <c r="B33" s="70" t="s">
-        <v>212</v>
-      </c>
-      <c r="C33" s="71" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A34" s="60"/>
-      <c r="B34" s="70" t="s">
-        <v>213</v>
-      </c>
-      <c r="C34" s="71"/>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A35" s="60"/>
-      <c r="B35" s="70" t="s">
-        <v>214</v>
-      </c>
-      <c r="C35" s="71"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A36" s="60"/>
-      <c r="B36" s="70" t="s">
-        <v>215</v>
-      </c>
-      <c r="C36" s="71"/>
-    </row>
-    <row r="37" spans="1:5" ht="32" x14ac:dyDescent="0.45">
-      <c r="A37" s="60"/>
-      <c r="B37" s="62" t="s">
-        <v>217</v>
-      </c>
-      <c r="C37" s="71"/>
-    </row>
-    <row r="38" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A38" s="60" t="s">
-        <v>238</v>
-      </c>
-      <c r="B38" s="70" t="s">
-        <v>218</v>
-      </c>
-      <c r="C38" s="71" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A39" s="60"/>
-      <c r="B39" s="70" t="s">
-        <v>219</v>
-      </c>
-      <c r="C39" s="71"/>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A40" s="60"/>
-      <c r="B40" s="70" t="s">
-        <v>220</v>
-      </c>
-      <c r="C40" s="71"/>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A42" s="72" t="s">
-        <v>288</v>
-      </c>
-      <c r="B42" s="73"/>
-      <c r="C42" s="74"/>
-    </row>
-    <row r="43" spans="1:5" ht="53" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A43" s="60" t="s">
-        <v>222</v>
-      </c>
-      <c r="B43" s="60"/>
-      <c r="C43" s="60"/>
-    </row>
-    <row r="44" spans="1:5" ht="50.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A44" s="60" t="s">
-        <v>223</v>
-      </c>
-      <c r="B44" s="60"/>
-      <c r="C44" s="60"/>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A46" s="59" t="s">
-        <v>287</v>
-      </c>
-      <c r="B46" s="59"/>
-      <c r="C46" s="59"/>
-      <c r="D46" s="59"/>
-      <c r="E46" s="59"/>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A47" s="55" t="s">
-        <v>239</v>
-      </c>
-      <c r="B47" s="55" t="s">
-        <v>248</v>
-      </c>
-      <c r="C47" s="55" t="s">
-        <v>249</v>
-      </c>
-      <c r="D47" s="55" t="s">
-        <v>250</v>
-      </c>
-      <c r="E47" s="55" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" ht="32" x14ac:dyDescent="0.45">
-      <c r="A48" s="53" t="s">
-        <v>252</v>
-      </c>
-      <c r="B48" s="53" t="s">
-        <v>240</v>
-      </c>
-      <c r="C48" s="53" t="s">
-        <v>253</v>
-      </c>
-      <c r="D48" s="53" t="s">
-        <v>241</v>
-      </c>
-      <c r="E48" s="53" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" ht="32" x14ac:dyDescent="0.45">
-      <c r="A49" s="53" t="s">
-        <v>254</v>
-      </c>
-      <c r="B49" s="53" t="s">
-        <v>243</v>
-      </c>
-      <c r="C49" s="53" t="s">
-        <v>255</v>
-      </c>
-      <c r="D49" s="53" t="s">
-        <v>241</v>
-      </c>
-      <c r="E49" s="53" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" ht="48" x14ac:dyDescent="0.45">
-      <c r="A50" s="53" t="s">
-        <v>256</v>
-      </c>
-      <c r="B50" s="53" t="s">
-        <v>243</v>
-      </c>
-      <c r="C50" s="53" t="s">
-        <v>257</v>
-      </c>
-      <c r="D50" s="53" t="s">
-        <v>244</v>
-      </c>
-      <c r="E50" s="53" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" ht="32" x14ac:dyDescent="0.45">
-      <c r="A51" s="53" t="s">
-        <v>259</v>
-      </c>
-      <c r="B51" s="53" t="s">
-        <v>245</v>
-      </c>
-      <c r="C51" s="53" t="s">
-        <v>260</v>
-      </c>
-      <c r="D51" s="53" t="s">
-        <v>246</v>
-      </c>
-      <c r="E51" s="53" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" ht="32" x14ac:dyDescent="0.45">
-      <c r="A52" s="53" t="s">
-        <v>261</v>
-      </c>
-      <c r="B52" s="53" t="s">
-        <v>245</v>
-      </c>
-      <c r="C52" s="53" t="s">
-        <v>262</v>
-      </c>
-      <c r="D52" s="53" t="s">
-        <v>246</v>
-      </c>
-      <c r="E52" s="53" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" ht="32" x14ac:dyDescent="0.45">
-      <c r="A53" s="53" t="s">
-        <v>263</v>
-      </c>
-      <c r="B53" s="53" t="s">
-        <v>245</v>
-      </c>
-      <c r="C53" s="53" t="s">
-        <v>264</v>
-      </c>
-      <c r="D53" s="53" t="s">
-        <v>247</v>
-      </c>
-      <c r="E53" s="53" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A54" s="53" t="s">
-        <v>265</v>
-      </c>
-      <c r="B54" s="53" t="s">
-        <v>245</v>
-      </c>
-      <c r="C54" s="53" t="s">
-        <v>266</v>
-      </c>
-      <c r="D54" s="53" t="s">
-        <v>241</v>
-      </c>
-      <c r="E54" s="53" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" ht="32" x14ac:dyDescent="0.45">
-      <c r="A55" s="53" t="s">
-        <v>267</v>
-      </c>
-      <c r="B55" s="53" t="s">
-        <v>245</v>
-      </c>
-      <c r="C55" s="53" t="s">
-        <v>268</v>
-      </c>
-      <c r="D55" s="53" t="s">
-        <v>247</v>
-      </c>
-      <c r="E55" s="53" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" ht="48" x14ac:dyDescent="0.45">
-      <c r="A56" s="53"/>
-      <c r="B56" s="54" t="s">
-        <v>270</v>
-      </c>
-      <c r="C56" s="54" t="s">
-        <v>272</v>
-      </c>
-      <c r="D56" s="54" t="s">
-        <v>273</v>
-      </c>
-      <c r="E56" s="75" t="s">
+      <c r="B59" s="83"/>
+      <c r="C59" s="84"/>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A60" s="53" t="s">
+        <v>292</v>
+      </c>
+      <c r="B60" s="53" t="s">
+        <v>293</v>
+      </c>
+      <c r="C60" s="53" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="32" x14ac:dyDescent="0.45">
+      <c r="A61" s="52" t="s">
+        <v>295</v>
+      </c>
+      <c r="B61" s="52" t="s">
+        <v>296</v>
+      </c>
+      <c r="C61" s="52" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="32" x14ac:dyDescent="0.45">
+      <c r="A62" s="52" t="s">
+        <v>298</v>
+      </c>
+      <c r="B62" s="52" t="s">
+        <v>299</v>
+      </c>
+      <c r="C62" s="52" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="32" x14ac:dyDescent="0.45">
+      <c r="A63" s="52" t="s">
+        <v>301</v>
+      </c>
+      <c r="B63" s="52" t="s">
+        <v>302</v>
+      </c>
+      <c r="C63" s="52" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A64" s="52" t="s">
+        <v>304</v>
+      </c>
+      <c r="B64" s="52" t="s">
+        <v>305</v>
+      </c>
+      <c r="C64" s="52" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A66" s="73" t="s">
+        <v>307</v>
+      </c>
+      <c r="B66" s="73"/>
+      <c r="C66" s="73"/>
+      <c r="D66" s="73"/>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A67" s="81" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" ht="48" x14ac:dyDescent="0.45">
-      <c r="A57" s="53"/>
-      <c r="B57" s="54" t="s">
-        <v>271</v>
-      </c>
-      <c r="C57" s="54" t="s">
-        <v>274</v>
-      </c>
-      <c r="D57" s="54" t="s">
-        <v>275</v>
-      </c>
-      <c r="E57" s="75" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A59" s="77" t="s">
-        <v>292</v>
-      </c>
-      <c r="B59" s="78"/>
-      <c r="C59" s="79"/>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A60" s="80" t="s">
-        <v>293</v>
-      </c>
-      <c r="B60" s="80" t="s">
-        <v>294</v>
-      </c>
-      <c r="C60" s="80" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" ht="32" x14ac:dyDescent="0.45">
-      <c r="A61" s="76" t="s">
-        <v>296</v>
-      </c>
-      <c r="B61" s="76" t="s">
-        <v>297</v>
-      </c>
-      <c r="C61" s="76" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" ht="32" x14ac:dyDescent="0.45">
-      <c r="A62" s="76" t="s">
-        <v>299</v>
-      </c>
-      <c r="B62" s="76" t="s">
-        <v>300</v>
-      </c>
-      <c r="C62" s="76" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" ht="32" x14ac:dyDescent="0.45">
-      <c r="A63" s="76" t="s">
-        <v>302</v>
-      </c>
-      <c r="B63" s="76" t="s">
-        <v>303</v>
-      </c>
-      <c r="C63" s="76" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A64" s="76" t="s">
-        <v>305</v>
-      </c>
-      <c r="B64" s="76" t="s">
-        <v>306</v>
-      </c>
-      <c r="C64" s="76" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A66" s="59" t="s">
-        <v>308</v>
-      </c>
-      <c r="B66" s="59"/>
-      <c r="C66" s="59"/>
-      <c r="D66" s="59"/>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A67" s="56" t="s">
+      <c r="B67" s="81"/>
+      <c r="C67" s="81"/>
+      <c r="D67" s="81"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A68" s="81" t="s">
         <v>277</v>
       </c>
-      <c r="B67" s="56"/>
-      <c r="C67" s="56"/>
-      <c r="D67" s="56"/>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A68" s="56" t="s">
+      <c r="B68" s="81"/>
+      <c r="C68" s="81"/>
+      <c r="D68" s="81"/>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A69" s="81" t="s">
         <v>278</v>
       </c>
-      <c r="B68" s="56"/>
-      <c r="C68" s="56"/>
-      <c r="D68" s="56"/>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A69" s="56" t="s">
+      <c r="B69" s="81"/>
+      <c r="C69" s="81"/>
+      <c r="D69" s="81"/>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A70" s="81" t="s">
         <v>279</v>
       </c>
-      <c r="B69" s="56"/>
-      <c r="C69" s="56"/>
-      <c r="D69" s="56"/>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A70" s="56" t="s">
+      <c r="B70" s="81"/>
+      <c r="C70" s="81"/>
+      <c r="D70" s="81"/>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A71" s="81" t="s">
         <v>280</v>
       </c>
-      <c r="B70" s="56"/>
-      <c r="C70" s="56"/>
-      <c r="D70" s="56"/>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A71" s="56" t="s">
+      <c r="B71" s="81"/>
+      <c r="C71" s="81"/>
+      <c r="D71" s="81"/>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A72" s="81" t="s">
         <v>281</v>
       </c>
-      <c r="B71" s="56"/>
-      <c r="C71" s="56"/>
-      <c r="D71" s="56"/>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A72" s="56" t="s">
+      <c r="B72" s="81"/>
+      <c r="C72" s="81"/>
+      <c r="D72" s="81"/>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A73" s="81" t="s">
         <v>282</v>
       </c>
-      <c r="B72" s="56"/>
-      <c r="C72" s="56"/>
-      <c r="D72" s="56"/>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A73" s="56" t="s">
+      <c r="B73" s="81"/>
+      <c r="C73" s="81"/>
+      <c r="D73" s="81"/>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A74" s="81" t="s">
         <v>283</v>
       </c>
-      <c r="B73" s="56"/>
-      <c r="C73" s="56"/>
-      <c r="D73" s="56"/>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A74" s="56" t="s">
+      <c r="B74" s="81"/>
+      <c r="C74" s="81"/>
+      <c r="D74" s="81"/>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A75" s="81" t="s">
         <v>284</v>
       </c>
-      <c r="B74" s="56"/>
-      <c r="C74" s="56"/>
-      <c r="D74" s="56"/>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A75" s="56" t="s">
-        <v>285</v>
-      </c>
-      <c r="B75" s="56"/>
-      <c r="C75" s="56"/>
-      <c r="D75" s="56"/>
+      <c r="B75" s="81"/>
+      <c r="C75" s="81"/>
+      <c r="D75" s="81"/>
     </row>
   </sheetData>
   <mergeCells count="25">
@@ -12782,11 +12656,6 @@
     <mergeCell ref="A70:D70"/>
     <mergeCell ref="A71:D71"/>
     <mergeCell ref="A72:D72"/>
-    <mergeCell ref="A38:A40"/>
-    <mergeCell ref="C38:C40"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A43:C43"/>
     <mergeCell ref="A44:C44"/>
     <mergeCell ref="A42:C42"/>
     <mergeCell ref="A32:C32"/>
@@ -12795,6 +12664,11 @@
     <mergeCell ref="A33:A37"/>
     <mergeCell ref="A31:C31"/>
     <mergeCell ref="A6:A10"/>
+    <mergeCell ref="A38:A40"/>
+    <mergeCell ref="C38:C40"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A43:C43"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>